<commit_message>
[ENH] Update saccade instructions to the shape-based cue
- Saccade/antisaccade instructions (ES/EN): the condition cue is now the shape (SQUARE = look at it, X = look to the opposite side) instead of the green/red ball

- Wording makes explicit that the stimulus is looked at while in the centre and the response starts when it moves to one of the sides

- BL2 (ES): prompt to press the central button to start
</commit_message>
<xml_diff>
--- a/src/instructions/module_1/[ES]BL2_instructions.xlsx
+++ b/src/instructions/module_1/[ES]BL2_instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\module_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{048CA441-B366-455D-9F61-12C919224A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2930AD7A-DAB8-435B-B7AD-4B6B4E082478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="4605" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>title</t>
   </si>
@@ -133,6 +133,9 @@
   <si>
     <t>El estímulo se mostrará durante 2 segundos.
 Responde lo mejor que puedas.</t>
+  </si>
+  <si>
+    <t>Pulsa el botón central para empezar la prueba.</t>
   </si>
 </sst>
 </file>
@@ -244,9 +247,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -284,7 +287,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -390,7 +393,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -532,7 +535,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -582,6 +585,9 @@
       <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -596,21 +602,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -724,30 +715,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -761,4 +744,27 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>